<commit_message>
Refresh sector data 2026-10-14
</commit_message>
<xml_diff>
--- a/backend/data/sectoraldata.xlsx
+++ b/backend/data/sectoraldata.xlsx
@@ -39399,7 +39399,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -39421,7 +39421,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -39443,7 +39443,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -39465,7 +39465,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -39487,7 +39487,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -39509,7 +39509,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -39531,7 +39531,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -39553,7 +39553,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -39575,7 +39575,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -39597,7 +39597,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -39619,7 +39619,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -39641,7 +39641,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -39663,7 +39663,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -39685,7 +39685,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -39707,7 +39707,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -39729,7 +39729,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -39751,7 +39751,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -39773,7 +39773,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -39795,7 +39795,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -39817,7 +39817,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -39839,7 +39839,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -39861,7 +39861,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -39883,7 +39883,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -39905,7 +39905,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -39927,7 +39927,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -39949,7 +39949,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -40007,7 +40007,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -40029,7 +40029,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -40051,7 +40051,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -40073,7 +40073,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -40095,7 +40095,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -40117,7 +40117,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -40139,7 +40139,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -40161,7 +40161,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -40183,7 +40183,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -40205,7 +40205,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -40227,7 +40227,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -40249,7 +40249,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -40271,7 +40271,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -40293,7 +40293,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -40315,7 +40315,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -40337,7 +40337,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -40359,7 +40359,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -40381,7 +40381,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -40403,7 +40403,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -40425,7 +40425,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -40447,7 +40447,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -40469,7 +40469,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -40491,7 +40491,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -40513,7 +40513,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -40535,7 +40535,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -40557,7 +40557,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">

</xml_diff>